<commit_message>
feat: Admin 王五 updated source data.xlsx
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yuhang/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778E0CE1-4C73-F045-A934-241C3ED39172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{83755A73-C422-6841-B77E-DBE23215E65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1584" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1577" uniqueCount="489">
   <si>
     <t>所在市</t>
   </si>
@@ -1443,12 +1443,6 @@
   </si>
   <si>
     <t>116.678255,39.908680</t>
-  </si>
-  <si>
-    <t>新光大中心5A</t>
-  </si>
-  <si>
-    <t>116.660425,39.916231</t>
   </si>
   <si>
     <t>Linda</t>
@@ -1882,7 +1876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B280671-4AFA-4641-88D4-A51F39483890}">
-  <dimension ref="A1:N193"/>
+  <dimension ref="A1:N192"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -1902,22 +1896,22 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1" t="s">
         <v>477</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>478</v>
+      </c>
+      <c r="D1" t="s">
         <v>479</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="F1" t="s">
         <v>480</v>
-      </c>
-      <c r="D1" t="s">
-        <v>481</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>487</v>
-      </c>
-      <c r="F1" t="s">
-        <v>482</v>
       </c>
       <c r="G1" t="s">
         <v>0</v>
@@ -1929,19 +1923,19 @@
         <v>2</v>
       </c>
       <c r="J1" t="s">
+        <v>481</v>
+      </c>
+      <c r="K1" t="s">
+        <v>476</v>
+      </c>
+      <c r="L1" t="s">
+        <v>482</v>
+      </c>
+      <c r="M1" t="s">
         <v>483</v>
       </c>
-      <c r="K1" t="s">
-        <v>478</v>
-      </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>484</v>
-      </c>
-      <c r="M1" t="s">
-        <v>485</v>
-      </c>
-      <c r="N1" t="s">
-        <v>486</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -1970,7 +1964,7 @@
         <v>9</v>
       </c>
       <c r="J2" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K2">
         <v>72308</v>
@@ -2011,7 +2005,7 @@
         <v>12</v>
       </c>
       <c r="J3" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K3">
         <v>72308</v>
@@ -2055,7 +2049,7 @@
         <v>17</v>
       </c>
       <c r="J4" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K4">
         <v>130769</v>
@@ -2099,7 +2093,7 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K5">
         <v>64615</v>
@@ -2143,7 +2137,7 @@
         <v>24</v>
       </c>
       <c r="J6" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K6">
         <v>80091</v>
@@ -2184,7 +2178,7 @@
         <v>27</v>
       </c>
       <c r="J7" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K7">
         <v>70673</v>
@@ -2228,7 +2222,7 @@
         <v>30</v>
       </c>
       <c r="J8" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K8">
         <v>90466</v>
@@ -2269,7 +2263,7 @@
         <v>32</v>
       </c>
       <c r="J9" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K9">
         <v>46720</v>
@@ -2313,7 +2307,7 @@
         <v>35</v>
       </c>
       <c r="J10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K10">
         <v>95000</v>
@@ -2357,7 +2351,7 @@
         <v>38</v>
       </c>
       <c r="J11" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K11">
         <v>85300</v>
@@ -2401,7 +2395,7 @@
         <v>41</v>
       </c>
       <c r="J12" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K12">
         <v>33305</v>
@@ -2445,7 +2439,7 @@
         <v>43</v>
       </c>
       <c r="J13" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K13">
         <v>120245.21</v>
@@ -2489,7 +2483,7 @@
         <v>43</v>
       </c>
       <c r="J14" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K14">
         <v>70425.53</v>
@@ -2533,7 +2527,7 @@
         <v>47</v>
       </c>
       <c r="J15" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K15">
         <v>78000</v>
@@ -2577,7 +2571,7 @@
         <v>50</v>
       </c>
       <c r="J16" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K16">
         <v>102796</v>
@@ -2621,7 +2615,7 @@
         <v>52</v>
       </c>
       <c r="J17" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K17">
         <v>49200</v>
@@ -2665,7 +2659,7 @@
         <v>54</v>
       </c>
       <c r="J18" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K18">
         <v>65096</v>
@@ -2709,7 +2703,7 @@
         <v>57</v>
       </c>
       <c r="J19" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K19">
         <v>56000</v>
@@ -2753,7 +2747,7 @@
         <v>60</v>
       </c>
       <c r="J20" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K20">
         <v>177847</v>
@@ -2797,7 +2791,7 @@
         <v>63</v>
       </c>
       <c r="J21" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K21">
         <v>83000</v>
@@ -2838,7 +2832,7 @@
         <v>66</v>
       </c>
       <c r="J22" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K22">
         <v>26000</v>
@@ -2879,7 +2873,7 @@
         <v>68</v>
       </c>
       <c r="J23" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K23">
         <v>85887</v>
@@ -2920,7 +2914,7 @@
         <v>70</v>
       </c>
       <c r="J24" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K24">
         <v>20000</v>
@@ -2964,7 +2958,7 @@
         <v>73</v>
       </c>
       <c r="J25" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K25">
         <v>146385</v>
@@ -3008,7 +3002,7 @@
         <v>76</v>
       </c>
       <c r="J26" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K26">
         <v>87000</v>
@@ -3052,7 +3046,7 @@
         <v>79</v>
       </c>
       <c r="J27" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K27">
         <v>147166.79999999999</v>
@@ -3096,7 +3090,7 @@
         <v>82</v>
       </c>
       <c r="J28" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K28">
         <v>46063</v>
@@ -3140,7 +3134,7 @@
         <v>85</v>
       </c>
       <c r="J29" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K29">
         <v>47261</v>
@@ -3184,7 +3178,7 @@
         <v>89</v>
       </c>
       <c r="J30" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K30">
         <v>119000</v>
@@ -3225,7 +3219,7 @@
         <v>92</v>
       </c>
       <c r="J31" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K31">
         <v>47000</v>
@@ -3269,7 +3263,7 @@
         <v>94</v>
       </c>
       <c r="J32" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K32">
         <v>186000</v>
@@ -3307,7 +3301,7 @@
         <v>96</v>
       </c>
       <c r="J33" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K33">
         <v>40800</v>
@@ -3348,7 +3342,7 @@
         <v>96</v>
       </c>
       <c r="J34" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K34">
         <v>55200</v>
@@ -3392,7 +3386,7 @@
         <v>100</v>
       </c>
       <c r="J35" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K35">
         <v>350000</v>
@@ -3433,7 +3427,7 @@
         <v>102</v>
       </c>
       <c r="J36" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K36">
         <v>65000</v>
@@ -3474,7 +3468,7 @@
         <v>102</v>
       </c>
       <c r="J37" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K37">
         <v>35000</v>
@@ -3515,7 +3509,7 @@
         <v>105</v>
       </c>
       <c r="J38" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K38">
         <v>47000</v>
@@ -3559,7 +3553,7 @@
         <v>108</v>
       </c>
       <c r="J39" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K39">
         <v>120000</v>
@@ -3600,7 +3594,7 @@
         <v>110</v>
       </c>
       <c r="J40" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K40">
         <v>83000</v>
@@ -3641,7 +3635,7 @@
         <v>112</v>
       </c>
       <c r="J41" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K41">
         <v>66030</v>
@@ -3679,7 +3673,7 @@
         <v>114</v>
       </c>
       <c r="J42" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K42">
         <v>40000</v>
@@ -3723,7 +3717,7 @@
         <v>119</v>
       </c>
       <c r="J43" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K43">
         <v>40000</v>
@@ -3764,7 +3758,7 @@
         <v>122</v>
       </c>
       <c r="J44" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K44">
         <v>54100</v>
@@ -3808,7 +3802,7 @@
         <v>125</v>
       </c>
       <c r="J45" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K45">
         <v>100000</v>
@@ -3852,7 +3846,7 @@
         <v>128</v>
       </c>
       <c r="J46" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K46">
         <v>150000</v>
@@ -3896,7 +3890,7 @@
         <v>131</v>
       </c>
       <c r="J47" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K47">
         <v>50000</v>
@@ -3940,7 +3934,7 @@
         <v>134</v>
       </c>
       <c r="J48" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K48">
         <v>43000</v>
@@ -3981,7 +3975,7 @@
         <v>137</v>
       </c>
       <c r="J49" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K49">
         <v>65000</v>
@@ -4022,7 +4016,7 @@
         <v>140</v>
       </c>
       <c r="J50" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -4054,7 +4048,7 @@
         <v>142</v>
       </c>
       <c r="J51" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K51">
         <v>56000</v>
@@ -4095,7 +4089,7 @@
         <v>144</v>
       </c>
       <c r="J52" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K52">
         <v>160000</v>
@@ -4136,7 +4130,7 @@
         <v>146</v>
       </c>
       <c r="J53" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K53">
         <v>33000</v>
@@ -4180,7 +4174,7 @@
         <v>149</v>
       </c>
       <c r="J54" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K54">
         <v>41318</v>
@@ -4221,7 +4215,7 @@
         <v>151</v>
       </c>
       <c r="J55" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K55">
         <v>34131</v>
@@ -4262,7 +4256,7 @@
         <v>154</v>
       </c>
       <c r="J56" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K56">
         <v>48000</v>
@@ -4303,7 +4297,7 @@
         <v>119</v>
       </c>
       <c r="J57" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K57">
         <v>16000</v>
@@ -4347,7 +4341,7 @@
         <v>158</v>
       </c>
       <c r="J58" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K58">
         <v>30000</v>
@@ -4391,7 +4385,7 @@
         <v>161</v>
       </c>
       <c r="J59" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K59">
         <v>56000</v>
@@ -4435,7 +4429,7 @@
         <v>164</v>
       </c>
       <c r="J60" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K60">
         <v>43000</v>
@@ -4476,7 +4470,7 @@
         <v>166</v>
       </c>
       <c r="J61" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K61">
         <v>110000</v>
@@ -4514,7 +4508,7 @@
         <v>168</v>
       </c>
       <c r="J62" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K62">
         <v>56160</v>
@@ -4555,7 +4549,7 @@
         <v>170</v>
       </c>
       <c r="J63" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K63">
         <v>138444</v>
@@ -4599,7 +4593,7 @@
         <v>174</v>
       </c>
       <c r="J64" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K64">
         <v>31000</v>
@@ -4640,7 +4634,7 @@
         <v>177</v>
       </c>
       <c r="J65" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K65">
         <v>120000</v>
@@ -4681,7 +4675,7 @@
         <v>179</v>
       </c>
       <c r="J66" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K66">
         <v>25900</v>
@@ -4722,7 +4716,7 @@
         <v>182</v>
       </c>
       <c r="J67" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K67">
         <v>47986</v>
@@ -4766,7 +4760,7 @@
         <v>184</v>
       </c>
       <c r="J68" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K68">
         <v>194000</v>
@@ -4810,7 +4804,7 @@
         <v>186</v>
       </c>
       <c r="J69" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K69">
         <v>39724</v>
@@ -4851,7 +4845,7 @@
         <v>188</v>
       </c>
       <c r="J70" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K70">
         <v>48437.45</v>
@@ -4892,7 +4886,7 @@
         <v>191</v>
       </c>
       <c r="J71" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K71">
         <v>37910</v>
@@ -4933,7 +4927,7 @@
         <v>193</v>
       </c>
       <c r="J72" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K72">
         <v>21220</v>
@@ -4974,7 +4968,7 @@
         <v>195</v>
       </c>
       <c r="J73" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K73">
         <v>77877</v>
@@ -5018,7 +5012,7 @@
         <v>197</v>
       </c>
       <c r="J74" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K74">
         <v>80311.53</v>
@@ -5062,7 +5056,7 @@
         <v>200</v>
       </c>
       <c r="J75" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K75">
         <v>38000</v>
@@ -5103,7 +5097,7 @@
         <v>203</v>
       </c>
       <c r="J76" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K76">
         <v>37800</v>
@@ -5147,7 +5141,7 @@
         <v>206</v>
       </c>
       <c r="J77" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K77">
         <v>54581</v>
@@ -5191,7 +5185,7 @@
         <v>89</v>
       </c>
       <c r="J78" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K78">
         <v>25000</v>
@@ -5235,7 +5229,7 @@
         <v>210</v>
       </c>
       <c r="J79" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K79">
         <v>52698</v>
@@ -5276,7 +5270,7 @@
         <v>214</v>
       </c>
       <c r="J80" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K80">
         <v>38500</v>
@@ -5314,7 +5308,7 @@
         <v>217</v>
       </c>
       <c r="J81" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="K81">
         <v>27200</v>
@@ -5358,7 +5352,7 @@
         <v>220</v>
       </c>
       <c r="J82" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K82">
         <v>60000</v>
@@ -5399,7 +5393,7 @@
         <v>223</v>
       </c>
       <c r="J83" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K83">
         <v>50000</v>
@@ -5443,7 +5437,7 @@
         <v>225</v>
       </c>
       <c r="J84" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K84">
         <v>131575</v>
@@ -5484,7 +5478,7 @@
         <v>227</v>
       </c>
       <c r="J85" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K85">
         <v>99500</v>
@@ -5525,7 +5519,7 @@
         <v>230</v>
       </c>
       <c r="J86" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K86">
         <v>32000</v>
@@ -5569,7 +5563,7 @@
         <v>232</v>
       </c>
       <c r="J87" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K87">
         <v>52170</v>
@@ -5610,7 +5604,7 @@
         <v>235</v>
       </c>
       <c r="J88" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K88">
         <v>46000</v>
@@ -5654,7 +5648,7 @@
         <v>238</v>
       </c>
       <c r="J89" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K89">
         <v>45013</v>
@@ -5695,7 +5689,7 @@
         <v>240</v>
       </c>
       <c r="J90" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K90">
         <v>48566</v>
@@ -5736,7 +5730,7 @@
         <v>243</v>
       </c>
       <c r="J91" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K91">
         <v>55618</v>
@@ -5777,7 +5771,7 @@
         <v>245</v>
       </c>
       <c r="J92" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K92">
         <v>47000</v>
@@ -5821,7 +5815,7 @@
         <v>248</v>
       </c>
       <c r="J93" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K93">
         <v>87763</v>
@@ -5865,7 +5859,7 @@
         <v>251</v>
       </c>
       <c r="J94" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K94">
         <v>100658</v>
@@ -5906,7 +5900,7 @@
         <v>254</v>
       </c>
       <c r="J95" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K95">
         <v>67000</v>
@@ -5950,7 +5944,7 @@
         <v>256</v>
       </c>
       <c r="J96" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K96">
         <v>39431</v>
@@ -5991,7 +5985,7 @@
         <v>258</v>
       </c>
       <c r="J97" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K97">
         <v>34273</v>
@@ -6029,7 +6023,7 @@
         <v>73</v>
       </c>
       <c r="J98" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K98">
         <v>40000</v>
@@ -6070,7 +6064,7 @@
         <v>261</v>
       </c>
       <c r="J99" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K99">
         <v>65000</v>
@@ -6114,7 +6108,7 @@
         <v>265</v>
       </c>
       <c r="J100" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="K100">
         <v>49000</v>
@@ -6158,7 +6152,7 @@
         <v>268</v>
       </c>
       <c r="J101" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="K101">
         <v>95000</v>
@@ -6202,7 +6196,7 @@
         <v>271</v>
       </c>
       <c r="J102" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="K102">
         <v>45000</v>
@@ -6243,7 +6237,7 @@
         <v>273</v>
       </c>
       <c r="J103" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="K103">
         <v>124500</v>
@@ -6284,7 +6278,7 @@
         <v>275</v>
       </c>
       <c r="J104" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="K104">
         <v>64000</v>
@@ -6325,7 +6319,7 @@
         <v>277</v>
       </c>
       <c r="J105" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="K105">
         <v>25000</v>
@@ -6366,7 +6360,7 @@
         <v>279</v>
       </c>
       <c r="J106" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="K106">
         <v>38498</v>
@@ -6404,7 +6398,7 @@
         <v>281</v>
       </c>
       <c r="J107" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K107">
         <v>166433</v>
@@ -6448,7 +6442,7 @@
         <v>283</v>
       </c>
       <c r="J108" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="K108">
         <v>58000</v>
@@ -6489,7 +6483,7 @@
         <v>286</v>
       </c>
       <c r="J109" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K109">
         <v>51872</v>
@@ -6530,7 +6524,7 @@
         <v>288</v>
       </c>
       <c r="J110" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K110">
         <v>21632</v>
@@ -6571,7 +6565,7 @@
         <v>290</v>
       </c>
       <c r="J111" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K111">
         <v>69000</v>
@@ -6612,7 +6606,7 @@
         <v>293</v>
       </c>
       <c r="J112" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K112">
         <v>54000</v>
@@ -6653,7 +6647,7 @@
         <v>295</v>
       </c>
       <c r="J113" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K113">
         <v>57400</v>
@@ -6694,7 +6688,7 @@
         <v>297</v>
       </c>
       <c r="J114" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K114">
         <v>60000</v>
@@ -6735,7 +6729,7 @@
         <v>297</v>
       </c>
       <c r="J115" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K115">
         <v>60000</v>
@@ -6773,7 +6767,7 @@
         <v>300</v>
       </c>
       <c r="J116" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K116">
         <v>33000</v>
@@ -6811,7 +6805,7 @@
         <v>302</v>
       </c>
       <c r="J117" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K117">
         <v>88786</v>
@@ -6849,7 +6843,7 @@
         <v>304</v>
       </c>
       <c r="J118" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K118">
         <v>134000</v>
@@ -6887,7 +6881,7 @@
         <v>306</v>
       </c>
       <c r="J119" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K119">
         <v>35000</v>
@@ -6925,7 +6919,7 @@
         <v>308</v>
       </c>
       <c r="J120" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K120">
         <v>18000</v>
@@ -6966,7 +6960,7 @@
         <v>310</v>
       </c>
       <c r="J121" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K121">
         <v>105741</v>
@@ -7004,7 +6998,7 @@
         <v>312</v>
       </c>
       <c r="J122" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K122">
         <v>51000</v>
@@ -7045,7 +7039,7 @@
         <v>314</v>
       </c>
       <c r="J123" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K123">
         <v>130143</v>
@@ -7080,7 +7074,7 @@
         <v>316</v>
       </c>
       <c r="J124" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K124">
         <v>121551.47</v>
@@ -7124,7 +7118,7 @@
         <v>320</v>
       </c>
       <c r="J125" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K125">
         <v>110000</v>
@@ -7168,7 +7162,7 @@
         <v>322</v>
       </c>
       <c r="J126" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K126">
         <v>56000</v>
@@ -7209,7 +7203,7 @@
         <v>324</v>
       </c>
       <c r="J127" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K127">
         <v>89177</v>
@@ -7253,7 +7247,7 @@
         <v>327</v>
       </c>
       <c r="J128" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K128">
         <v>30000</v>
@@ -7297,7 +7291,7 @@
         <v>329</v>
       </c>
       <c r="J129" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K129">
         <v>54550</v>
@@ -7341,7 +7335,7 @@
         <v>331</v>
       </c>
       <c r="J130" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K130">
         <v>125000</v>
@@ -7385,7 +7379,7 @@
         <v>334</v>
       </c>
       <c r="J131" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K131">
         <v>69100</v>
@@ -7429,7 +7423,7 @@
         <v>336</v>
       </c>
       <c r="J132" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K132">
         <v>118290</v>
@@ -7470,7 +7464,7 @@
         <v>339</v>
       </c>
       <c r="J133" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K133">
         <v>79900</v>
@@ -7511,7 +7505,7 @@
         <v>341</v>
       </c>
       <c r="J134" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K134">
         <v>39742.379999999997</v>
@@ -7555,7 +7549,7 @@
         <v>343</v>
       </c>
       <c r="J135" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K135">
         <v>48000</v>
@@ -7596,7 +7590,7 @@
         <v>345</v>
       </c>
       <c r="J136" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K136">
         <v>74722</v>
@@ -7634,7 +7628,7 @@
         <v>347</v>
       </c>
       <c r="J137" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K137">
         <v>55000</v>
@@ -7672,7 +7666,7 @@
         <v>350</v>
       </c>
       <c r="J138" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K138">
         <v>128000</v>
@@ -7716,7 +7710,7 @@
         <v>352</v>
       </c>
       <c r="J139" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K139">
         <v>122000</v>
@@ -7757,7 +7751,7 @@
         <v>354</v>
       </c>
       <c r="J140" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K140">
         <v>22000</v>
@@ -7798,7 +7792,7 @@
         <v>356</v>
       </c>
       <c r="J141" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K141">
         <v>10000</v>
@@ -7839,7 +7833,7 @@
         <v>358</v>
       </c>
       <c r="J142" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K142">
         <v>64000</v>
@@ -7880,7 +7874,7 @@
         <v>360</v>
       </c>
       <c r="J143" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K143">
         <v>95628</v>
@@ -7921,7 +7915,7 @@
         <v>363</v>
       </c>
       <c r="J144" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K144">
         <v>39562</v>
@@ -7965,7 +7959,7 @@
         <v>366</v>
       </c>
       <c r="J145" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K145">
         <v>105000</v>
@@ -8009,7 +8003,7 @@
         <v>368</v>
       </c>
       <c r="J146" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K146">
         <v>60000</v>
@@ -8050,7 +8044,7 @@
         <v>370</v>
       </c>
       <c r="J147" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K147">
         <v>39964</v>
@@ -8091,7 +8085,7 @@
         <v>372</v>
       </c>
       <c r="J148" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K148">
         <v>94000</v>
@@ -8135,7 +8129,7 @@
         <v>368</v>
       </c>
       <c r="J149" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K149">
         <v>75000</v>
@@ -8176,7 +8170,7 @@
         <v>188</v>
       </c>
       <c r="J150" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K150">
         <v>48767</v>
@@ -8220,7 +8214,7 @@
         <v>376</v>
       </c>
       <c r="J151" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K151">
         <v>63824</v>
@@ -8264,7 +8258,7 @@
         <v>378</v>
       </c>
       <c r="J152" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K152">
         <v>117000</v>
@@ -8302,7 +8296,7 @@
         <v>380</v>
       </c>
       <c r="J153" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K153">
         <v>41000</v>
@@ -8340,7 +8334,7 @@
         <v>382</v>
       </c>
       <c r="J154" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K154">
         <v>96446</v>
@@ -8384,7 +8378,7 @@
         <v>386</v>
       </c>
       <c r="J155" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K155">
         <v>76600</v>
@@ -8425,7 +8419,7 @@
         <v>388</v>
       </c>
       <c r="J156" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K156">
         <v>125569</v>
@@ -8466,7 +8460,7 @@
         <v>391</v>
       </c>
       <c r="J157" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K157">
         <v>51234</v>
@@ -8510,7 +8504,7 @@
         <v>393</v>
       </c>
       <c r="J158" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K158">
         <v>123780</v>
@@ -8551,7 +8545,7 @@
         <v>396</v>
       </c>
       <c r="J159" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K159">
         <v>46000</v>
@@ -8589,7 +8583,7 @@
         <v>398</v>
       </c>
       <c r="J160" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K160">
         <v>35600</v>
@@ -8630,7 +8624,7 @@
         <v>400</v>
       </c>
       <c r="J161" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K161">
         <v>199950</v>
@@ -8671,7 +8665,7 @@
         <v>402</v>
       </c>
       <c r="J162" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K162">
         <v>108000</v>
@@ -8712,7 +8706,7 @@
         <v>404</v>
       </c>
       <c r="J163" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K163">
         <v>142808</v>
@@ -8753,7 +8747,7 @@
         <v>406</v>
       </c>
       <c r="J164" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K164">
         <v>80463</v>
@@ -8794,7 +8788,7 @@
         <v>408</v>
       </c>
       <c r="J165" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K165">
         <v>83000</v>
@@ -8832,7 +8826,7 @@
         <v>410</v>
       </c>
       <c r="J166" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K166">
         <v>129000</v>
@@ -8873,7 +8867,7 @@
         <v>413</v>
       </c>
       <c r="J167" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K167">
         <v>62209</v>
@@ -8914,7 +8908,7 @@
         <v>415</v>
       </c>
       <c r="J168" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K168">
         <v>36117</v>
@@ -8958,7 +8952,7 @@
         <v>417</v>
       </c>
       <c r="J169" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K169">
         <v>49900</v>
@@ -9002,7 +8996,7 @@
         <v>420</v>
       </c>
       <c r="J170" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K170">
         <v>39000</v>
@@ -9043,7 +9037,7 @@
         <v>422</v>
       </c>
       <c r="J171" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K171">
         <v>49000</v>
@@ -9081,7 +9075,7 @@
         <v>424</v>
       </c>
       <c r="J172" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K172">
         <v>59400</v>
@@ -9122,7 +9116,7 @@
         <v>426</v>
       </c>
       <c r="J173" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K173">
         <v>65000</v>
@@ -9166,7 +9160,7 @@
         <v>431</v>
       </c>
       <c r="J174" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K174">
         <v>47000</v>
@@ -9207,7 +9201,7 @@
         <v>433</v>
       </c>
       <c r="J175" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K175">
         <v>29000</v>
@@ -9251,7 +9245,7 @@
         <v>435</v>
       </c>
       <c r="J176" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K176">
         <v>132239</v>
@@ -9292,7 +9286,7 @@
         <v>437</v>
       </c>
       <c r="J177" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K177">
         <v>35016</v>
@@ -9330,7 +9324,7 @@
         <v>439</v>
       </c>
       <c r="J178" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K178">
         <v>60000</v>
@@ -9371,7 +9365,7 @@
         <v>442</v>
       </c>
       <c r="J179" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K179">
         <v>90244</v>
@@ -9409,7 +9403,7 @@
         <v>444</v>
       </c>
       <c r="J180" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K180">
         <v>38700</v>
@@ -9447,7 +9441,7 @@
         <v>446</v>
       </c>
       <c r="J181" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K181">
         <v>62414</v>
@@ -9485,7 +9479,7 @@
         <v>448</v>
       </c>
       <c r="J182" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K182">
         <v>51000</v>
@@ -9526,7 +9520,7 @@
         <v>450</v>
       </c>
       <c r="J183" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K183">
         <v>53115</v>
@@ -9564,7 +9558,7 @@
         <v>452</v>
       </c>
       <c r="J184" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K184">
         <v>120000</v>
@@ -9605,7 +9599,7 @@
         <v>454</v>
       </c>
       <c r="J185" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K185">
         <v>66477</v>
@@ -9872,44 +9866,6 @@
       </c>
       <c r="N192">
         <v>15800</v>
-      </c>
-    </row>
-    <row r="193" spans="1:14">
-      <c r="A193">
-        <v>192</v>
-      </c>
-      <c r="B193" t="s">
-        <v>470</v>
-      </c>
-      <c r="C193" t="s">
-        <v>456</v>
-      </c>
-      <c r="D193" t="s">
-        <v>5</v>
-      </c>
-      <c r="E193" t="s">
-        <v>16</v>
-      </c>
-      <c r="G193" t="s">
-        <v>7</v>
-      </c>
-      <c r="H193" t="s">
-        <v>457</v>
-      </c>
-      <c r="I193" t="s">
-        <v>471</v>
-      </c>
-      <c r="K193">
-        <v>76210</v>
-      </c>
-      <c r="L193">
-        <v>84.4444444444444</v>
-      </c>
-      <c r="M193">
-        <v>0.38052748983073098</v>
-      </c>
-      <c r="N193">
-        <v>29000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Admin 王五 updated data.xlsx
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\intern.bjres\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4D5EC1-FCC0-42F2-9F57-D68676696921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4418A411-CD78-437E-8C54-3AB01827D95B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="45" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="451">
   <si>
     <t>所在市</t>
   </si>
@@ -1384,6 +1384,9 @@
   </si>
   <si>
     <t>上季度免租期</t>
+  </si>
+  <si>
+    <t>116.680295,39.907589</t>
   </si>
 </sst>
 </file>
@@ -1467,10 +1470,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -12068,7 +12067,7 @@
         <v>66</v>
       </c>
       <c r="I190" t="s">
-        <v>67</v>
+        <v>450</v>
       </c>
       <c r="K190">
         <v>26737</v>

</xml_diff>